<commit_message>
pytest_Anatomy files, added column 'area'
</commit_message>
<xml_diff>
--- a/tests/config_files/pytest_Anatomy_config.xlsx
+++ b/tests/config_files/pytest_Anatomy_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\opt2\Git_Repos\CxSystem2\tests\config_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\opt2\git_repos\CxSystem2\tests\config_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F614EAD-2B74-4504-8C86-D0A10F06F0E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10062505-20D0-412B-8A87-611B4F7E840C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{7826B0A7-9CAB-4844-8FAC-668DF56D5877}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7826B0A7-9CAB-4844-8FAC-668DF56D5877}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="173">
   <si>
     <t>row_type</t>
   </si>
@@ -558,6 +558,12 @@
   </si>
   <si>
     <t>./tests/connection_files/sim_pytest_connections_20240731_1413026.gz</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>V1</t>
   </si>
 </sst>
 </file>
@@ -1449,46 +1455,46 @@
         <v>27</v>
       </c>
       <c r="C8" t="s">
+        <v>171</v>
+      </c>
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>40</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>41</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>42</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>32</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>33</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>43</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>44</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>45</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>46</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>47</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>48</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>49</v>
-      </c>
-      <c r="P8" t="s">
-        <v>24</v>
       </c>
       <c r="Q8" t="s">
         <v>24</v>
@@ -1505,32 +1511,32 @@
         <v>20</v>
       </c>
       <c r="C9" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" t="s">
         <v>52</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>53</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>54</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>55</v>
       </c>
-      <c r="G9" t="s">
-        <v>56</v>
-      </c>
       <c r="H9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I9" t="s">
         <v>39</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>57</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>58</v>
       </c>
-      <c r="K9" t="s">
-        <v>56</v>
-      </c>
       <c r="L9" t="s">
         <v>56</v>
       </c>
@@ -1544,7 +1550,7 @@
         <v>56</v>
       </c>
       <c r="P9" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Q9" t="s">
         <v>24</v>
@@ -1561,32 +1567,32 @@
         <v>144</v>
       </c>
       <c r="C10" t="s">
+        <v>172</v>
+      </c>
+      <c r="D10" t="s">
         <v>59</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>60</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>55</v>
       </c>
-      <c r="G10" t="s">
-        <v>56</v>
-      </c>
       <c r="H10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" t="s">
         <v>39</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>57</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>58</v>
       </c>
-      <c r="K10" t="s">
-        <v>56</v>
-      </c>
       <c r="L10" t="s">
         <v>56</v>
       </c>
@@ -1600,7 +1606,7 @@
         <v>56</v>
       </c>
       <c r="P10" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Q10" t="s">
         <v>24</v>
@@ -1617,32 +1623,32 @@
         <v>132</v>
       </c>
       <c r="C11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" t="s">
         <v>62</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>63</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>64</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>65</v>
       </c>
-      <c r="G11" t="s">
-        <v>56</v>
-      </c>
       <c r="H11" t="s">
+        <v>56</v>
+      </c>
+      <c r="I11" t="s">
         <v>39</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>57</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>58</v>
       </c>
-      <c r="K11" t="s">
-        <v>56</v>
-      </c>
       <c r="L11" t="s">
         <v>56</v>
       </c>
@@ -1656,7 +1662,7 @@
         <v>56</v>
       </c>
       <c r="P11" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Q11" t="s">
         <v>24</v>
@@ -1673,32 +1679,32 @@
         <v>65</v>
       </c>
       <c r="C12" t="s">
+        <v>172</v>
+      </c>
+      <c r="D12" t="s">
         <v>67</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>69</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>65</v>
       </c>
-      <c r="G12" t="s">
-        <v>56</v>
-      </c>
       <c r="H12" t="s">
+        <v>56</v>
+      </c>
+      <c r="I12" t="s">
         <v>39</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>70</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>71</v>
       </c>
-      <c r="K12" t="s">
-        <v>56</v>
-      </c>
       <c r="L12" t="s">
         <v>56</v>
       </c>
@@ -1712,7 +1718,7 @@
         <v>56</v>
       </c>
       <c r="P12" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Q12" t="s">
         <v>24</v>
@@ -1729,32 +1735,32 @@
         <v>51</v>
       </c>
       <c r="C13" t="s">
+        <v>172</v>
+      </c>
+      <c r="D13" t="s">
         <v>73</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>74</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>75</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>65</v>
       </c>
-      <c r="G13" t="s">
-        <v>56</v>
-      </c>
       <c r="H13" t="s">
+        <v>56</v>
+      </c>
+      <c r="I13" t="s">
         <v>39</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>70</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>71</v>
       </c>
-      <c r="K13" t="s">
-        <v>56</v>
-      </c>
       <c r="L13" t="s">
         <v>56</v>
       </c>
@@ -1768,7 +1774,7 @@
         <v>56</v>
       </c>
       <c r="P13" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="Q13" t="s">
         <v>24</v>
@@ -1782,9 +1788,6 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" t="s">
         <v>24</v>
       </c>
       <c r="D14" t="s">

</xml_diff>